<commit_message>
chore: 更新 CheckList 模板
Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/CheckList模板.xlsx
+++ b/CheckList模板.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowHeight="15160"/>
+    <workbookView windowHeight="16660"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="312" uniqueCount="90">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="318" uniqueCount="89">
   <si>
     <t>类型</t>
   </si>
@@ -114,9 +114,6 @@
   </si>
   <si>
     <t>检查OTA部署表文档真实存在即可，或者文本描述存在"无断开"的描述都通过；还有就是文本描述"有断开"，且说明原因，则通过</t>
-  </si>
-  <si>
-    <t>同上</t>
   </si>
   <si>
     <t>确认历史版本是否全市场推送，如有特殊市场未推OTA，备注中说明原因</t>
@@ -1318,7 +1315,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="19">
+  <cellXfs count="20">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1355,6 +1352,9 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="4" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -1374,7 +1374,7 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -2068,7 +2068,7 @@
       </c>
     </row>
     <row r="9" ht="41" spans="1:6">
-      <c r="A9" s="8" t="s">
+      <c r="A9" s="12" t="s">
         <v>6</v>
       </c>
       <c r="B9" s="9" t="s">
@@ -2087,8 +2087,10 @@
         <v>28</v>
       </c>
     </row>
-    <row r="10" ht="28" spans="1:6">
-      <c r="A10" s="8"/>
+    <row r="10" ht="41" spans="1:6">
+      <c r="A10" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="B10" s="9" t="s">
         <v>24</v>
       </c>
@@ -2102,15 +2104,15 @@
         <v>10</v>
       </c>
       <c r="F10" s="7" t="s">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="11" ht="55" spans="1:6">
+      <c r="A11" s="12" t="s">
+        <v>6</v>
+      </c>
+      <c r="B11" s="9" t="s">
         <v>29</v>
-      </c>
-    </row>
-    <row r="11" ht="55" spans="1:6">
-      <c r="A11" s="8" t="s">
-        <v>6</v>
-      </c>
-      <c r="B11" s="9" t="s">
-        <v>30</v>
       </c>
       <c r="C11" s="5" t="s">
         <v>25</v>
@@ -2122,13 +2124,15 @@
         <v>27</v>
       </c>
       <c r="F11" s="7" t="s">
-        <v>31</v>
-      </c>
-    </row>
-    <row r="12" ht="28" spans="1:6">
-      <c r="A12" s="8"/>
+        <v>30</v>
+      </c>
+    </row>
+    <row r="12" ht="55" spans="1:6">
+      <c r="A12" s="12" t="s">
+        <v>6</v>
+      </c>
       <c r="B12" s="9" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
       <c r="C12" s="5" t="s">
         <v>8</v>
@@ -2140,75 +2144,75 @@
         <v>10</v>
       </c>
       <c r="F12" s="7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
     </row>
     <row r="13" ht="136" spans="1:6">
       <c r="A13" s="8" t="s">
+        <v>31</v>
+      </c>
+      <c r="B13" s="9" t="s">
         <v>32</v>
       </c>
-      <c r="B13" s="9" t="s">
+      <c r="C13" s="5" t="s">
         <v>33</v>
       </c>
-      <c r="C13" s="5" t="s">
+      <c r="D13" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D13" s="6" t="s">
+      <c r="E13" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E13" s="6" t="s">
+      <c r="F13" s="7" t="s">
         <v>36</v>
-      </c>
-      <c r="F13" s="7" t="s">
-        <v>37</v>
       </c>
     </row>
     <row r="14" ht="204" spans="1:6">
       <c r="A14" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B14" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B14" s="13" t="s">
+        <v>37</v>
+      </c>
+      <c r="C14" s="5" t="s">
         <v>38</v>
       </c>
-      <c r="C14" s="5" t="s">
+      <c r="D14" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D14" s="6" t="s">
+      <c r="E14" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E14" s="6" t="s">
+      <c r="F14" s="7" t="s">
         <v>41</v>
-      </c>
-      <c r="F14" s="7" t="s">
-        <v>42</v>
       </c>
     </row>
     <row r="15" ht="123" spans="1:6">
       <c r="A15" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B15" s="10" t="s">
+        <v>42</v>
+      </c>
+      <c r="C15" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D15" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E15" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F15" s="7" t="s">
         <v>43</v>
-      </c>
-      <c r="C15" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D15" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E15" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F15" s="7" t="s">
-        <v>44</v>
       </c>
     </row>
     <row r="16" ht="164" spans="1:6">
       <c r="A16" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B16" s="10" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C16" s="5" t="s">
         <v>25</v>
@@ -2220,15 +2224,15 @@
         <v>27</v>
       </c>
       <c r="F16" s="7" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
     </row>
     <row r="17" ht="354" spans="1:6">
       <c r="A17" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B17" s="10" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C17" s="5" t="s">
         <v>25</v>
@@ -2240,15 +2244,15 @@
         <v>27</v>
       </c>
       <c r="F17" s="7" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
     </row>
     <row r="18" ht="313" spans="1:6">
       <c r="A18" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B18" s="9" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C18" s="5" t="s">
         <v>8</v>
@@ -2260,15 +2264,15 @@
         <v>10</v>
       </c>
       <c r="F18" s="7" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
     </row>
     <row r="19" ht="245" spans="1:6">
       <c r="A19" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B19" s="9" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C19" s="5" t="s">
         <v>8</v>
@@ -2280,15 +2284,15 @@
         <v>10</v>
       </c>
       <c r="F19" s="7" t="s">
+        <v>51</v>
+      </c>
+    </row>
+    <row r="20" ht="164" spans="1:6">
+      <c r="A20" s="12" t="s">
+        <v>31</v>
+      </c>
+      <c r="B20" s="10" t="s">
         <v>52</v>
-      </c>
-    </row>
-    <row r="20" ht="164" spans="1:6">
-      <c r="A20" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B20" s="10" t="s">
-        <v>53</v>
       </c>
       <c r="C20" s="5" t="s">
         <v>25</v>
@@ -2300,51 +2304,55 @@
         <v>27</v>
       </c>
       <c r="F20" s="7" t="s">
-        <v>54</v>
-      </c>
-    </row>
-    <row r="21" ht="68" spans="1:6">
-      <c r="A21" s="8"/>
+        <v>53</v>
+      </c>
+    </row>
+    <row r="21" ht="164" spans="1:6">
+      <c r="A21" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="B21" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D21" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E21" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F21" s="7" t="s">
         <v>53</v>
       </c>
-      <c r="C21" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D21" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E21" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F21" s="7" t="s">
-        <v>29</v>
-      </c>
-    </row>
-    <row r="22" ht="68" spans="1:6">
-      <c r="A22" s="8"/>
+    </row>
+    <row r="22" ht="164" spans="1:6">
+      <c r="A22" s="12" t="s">
+        <v>31</v>
+      </c>
       <c r="B22" s="10" t="s">
+        <v>52</v>
+      </c>
+      <c r="C22" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D22" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E22" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F22" s="7" t="s">
         <v>53</v>
-      </c>
-      <c r="C22" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D22" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E22" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F22" s="7" t="s">
-        <v>29</v>
       </c>
     </row>
     <row r="23" ht="123" spans="1:6">
       <c r="A23" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B23" s="9" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C23" s="5" t="s">
         <v>25</v>
@@ -2356,15 +2364,15 @@
         <v>27</v>
       </c>
       <c r="F23" s="7" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
     </row>
     <row r="24" ht="272" spans="1:6">
       <c r="A24" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B24" s="9" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>25</v>
@@ -2376,15 +2384,15 @@
         <v>27</v>
       </c>
       <c r="F24" s="7" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="25" ht="300" spans="1:6">
       <c r="A25" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B25" s="9" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>8</v>
@@ -2396,15 +2404,15 @@
         <v>10</v>
       </c>
       <c r="F25" s="7" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="26" ht="409.5" spans="1:6">
       <c r="A26" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B26" s="9" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>8</v>
@@ -2416,15 +2424,15 @@
         <v>10</v>
       </c>
       <c r="F26" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="27" ht="409.5" spans="1:6">
       <c r="A27" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B27" s="13" t="s">
-        <v>63</v>
+        <v>31</v>
+      </c>
+      <c r="B27" s="14" t="s">
+        <v>62</v>
       </c>
       <c r="C27" s="5" t="s">
         <v>8</v>
@@ -2436,15 +2444,15 @@
         <v>10</v>
       </c>
       <c r="F27" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="28" ht="409.5" spans="1:6">
       <c r="A28" s="8" t="s">
-        <v>32</v>
-      </c>
-      <c r="B28" s="13" t="s">
-        <v>64</v>
+        <v>31</v>
+      </c>
+      <c r="B28" s="14" t="s">
+        <v>63</v>
       </c>
       <c r="C28" s="5" t="s">
         <v>8</v>
@@ -2456,15 +2464,15 @@
         <v>10</v>
       </c>
       <c r="F28" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="29" ht="409.5" spans="1:6">
       <c r="A29" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B29" s="9" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C29" s="5" t="s">
         <v>8</v>
@@ -2476,15 +2484,15 @@
         <v>10</v>
       </c>
       <c r="F29" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="30" ht="409.5" spans="1:6">
       <c r="A30" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B30" s="9" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C30" s="5" t="s">
         <v>8</v>
@@ -2496,15 +2504,15 @@
         <v>10</v>
       </c>
       <c r="F30" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="31" ht="409.5" spans="1:6">
       <c r="A31" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B31" s="9" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C31" s="5" t="s">
         <v>8</v>
@@ -2516,15 +2524,15 @@
         <v>10</v>
       </c>
       <c r="F31" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="32" ht="409.5" spans="1:6">
       <c r="A32" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B32" s="9" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C32" s="5" t="s">
         <v>8</v>
@@ -2536,15 +2544,15 @@
         <v>10</v>
       </c>
       <c r="F32" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="33" ht="409.5" spans="1:6">
       <c r="A33" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B33" s="9" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C33" s="5" t="s">
         <v>8</v>
@@ -2556,15 +2564,15 @@
         <v>10</v>
       </c>
       <c r="F33" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="34" ht="409.5" spans="1:6">
       <c r="A34" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B34" s="9" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C34" s="5" t="s">
         <v>8</v>
@@ -2576,15 +2584,15 @@
         <v>10</v>
       </c>
       <c r="F34" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="35" ht="409.5" spans="1:6">
       <c r="A35" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B35" s="9" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C35" s="5" t="s">
         <v>8</v>
@@ -2596,15 +2604,15 @@
         <v>10</v>
       </c>
       <c r="F35" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="36" ht="409.5" spans="1:6">
       <c r="A36" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B36" s="9" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C36" s="5" t="s">
         <v>8</v>
@@ -2616,15 +2624,15 @@
         <v>10</v>
       </c>
       <c r="F36" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="37" ht="409.5" spans="1:6">
       <c r="A37" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B37" s="9" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>8</v>
@@ -2636,15 +2644,15 @@
         <v>10</v>
       </c>
       <c r="F37" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="38" ht="409.5" spans="1:6">
       <c r="A38" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B38" s="9" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C38" s="5" t="s">
         <v>8</v>
@@ -2656,195 +2664,195 @@
         <v>10</v>
       </c>
       <c r="F38" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="39" ht="409.5" spans="1:6">
       <c r="A39" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B39" s="9" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C39" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D39" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D39" s="6" t="s">
+      <c r="E39" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E39" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F39" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="40" ht="409.5" spans="1:6">
       <c r="A40" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B40" s="9" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C40" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D40" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D40" s="6" t="s">
+      <c r="E40" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E40" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F40" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="41" ht="409.5" spans="1:6">
       <c r="A41" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B41" s="9" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C41" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D41" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D41" s="6" t="s">
+      <c r="E41" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E41" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F41" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="42" ht="409.5" spans="1:6">
       <c r="A42" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B42" s="9" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C42" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D42" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D42" s="6" t="s">
+      <c r="E42" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E42" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F42" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="43" ht="409.5" spans="1:6">
       <c r="A43" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B43" s="9" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C43" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D43" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D43" s="6" t="s">
+      <c r="E43" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E43" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F43" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="44" ht="409.5" spans="1:6">
       <c r="A44" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B44" s="9" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C44" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D44" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D44" s="6" t="s">
+      <c r="E44" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E44" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F44" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="45" ht="409.5" spans="1:6">
       <c r="A45" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B45" s="9" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C45" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D45" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D45" s="6" t="s">
+      <c r="E45" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E45" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F45" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="46" ht="409.5" spans="1:6">
       <c r="A46" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B46" s="9" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C46" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D46" s="6" t="s">
         <v>34</v>
       </c>
-      <c r="D46" s="6" t="s">
+      <c r="E46" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="E46" s="6" t="s">
-        <v>36</v>
-      </c>
       <c r="F46" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="47" ht="409.5" spans="1:6">
       <c r="A47" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B47" s="9" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C47" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D47" s="6" t="s">
         <v>39</v>
       </c>
-      <c r="D47" s="6" t="s">
+      <c r="E47" s="6" t="s">
         <v>40</v>
       </c>
-      <c r="E47" s="6" t="s">
-        <v>41</v>
-      </c>
       <c r="F47" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" ht="409.5" spans="1:6">
       <c r="A48" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B48" s="9" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>25</v>
@@ -2856,15 +2864,15 @@
         <v>27</v>
       </c>
       <c r="F48" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="49" ht="409.5" spans="1:6">
       <c r="A49" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B49" s="9" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>25</v>
@@ -2876,15 +2884,15 @@
         <v>27</v>
       </c>
       <c r="F49" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="50" ht="409.5" spans="1:6">
       <c r="A50" s="8" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="B50" s="9" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C50" s="5" t="s">
         <v>25</v>
@@ -2896,73 +2904,70 @@
         <v>27</v>
       </c>
       <c r="F50" s="7" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
     </row>
     <row r="51" ht="409.5" spans="1:6">
-      <c r="A51" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="B51" s="15" t="s">
+      <c r="A51" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="B51" s="16" t="s">
+        <v>86</v>
+      </c>
+      <c r="C51" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="D51" s="18" t="s">
+        <v>26</v>
+      </c>
+      <c r="E51" s="18" t="s">
+        <v>27</v>
+      </c>
+      <c r="F51" s="7" t="s">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="52" ht="191" spans="1:6">
+      <c r="A52" s="19" t="s">
+        <v>6</v>
+      </c>
+      <c r="B52" s="19" t="s">
         <v>87</v>
       </c>
-      <c r="C51" s="16" t="s">
-        <v>25</v>
-      </c>
-      <c r="D51" s="17" t="s">
-        <v>26</v>
-      </c>
-      <c r="E51" s="17" t="s">
-        <v>27</v>
-      </c>
-      <c r="F51" s="7" t="s">
-        <v>62</v>
-      </c>
-    </row>
-    <row r="52" ht="191" spans="1:6">
-      <c r="A52" s="5" t="s">
+      <c r="C52" s="5" t="s">
+        <v>33</v>
+      </c>
+      <c r="D52" s="6" t="s">
+        <v>34</v>
+      </c>
+      <c r="E52" s="6" t="s">
+        <v>35</v>
+      </c>
+      <c r="F52" s="7" t="s">
+        <v>88</v>
+      </c>
+    </row>
+    <row r="53" ht="191" spans="1:6">
+      <c r="A53" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="B52" s="18" t="s">
+      <c r="B53" s="19" t="s">
+        <v>87</v>
+      </c>
+      <c r="C53" s="5" t="s">
+        <v>38</v>
+      </c>
+      <c r="D53" s="6" t="s">
+        <v>39</v>
+      </c>
+      <c r="E53" s="6" t="s">
+        <v>40</v>
+      </c>
+      <c r="F53" s="7" t="s">
         <v>88</v>
       </c>
-      <c r="C52" s="5" t="s">
-        <v>34</v>
-      </c>
-      <c r="D52" s="6" t="s">
-        <v>35</v>
-      </c>
-      <c r="E52" s="6" t="s">
-        <v>36</v>
-      </c>
-      <c r="F52" s="7" t="s">
-        <v>89</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6">
-      <c r="A53" s="5"/>
-      <c r="B53" s="18"/>
-      <c r="C53" s="5" t="s">
-        <v>39</v>
-      </c>
-      <c r="D53" s="6" t="s">
-        <v>40</v>
-      </c>
-      <c r="E53" s="6" t="s">
-        <v>41</v>
-      </c>
-      <c r="F53" s="7" t="s">
-        <v>29</v>
-      </c>
     </row>
   </sheetData>
-  <mergeCells count="5">
-    <mergeCell ref="A9:A10"/>
-    <mergeCell ref="A11:A12"/>
-    <mergeCell ref="A20:A22"/>
-    <mergeCell ref="A52:A53"/>
-    <mergeCell ref="B52:B53"/>
-  </mergeCells>
   <dataValidations count="4">
     <dataValidation allowBlank="1" showInputMessage="1" showErrorMessage="1" sqref="C2:D2 D10 D12 D3:D8 D18:D19 D25:D38"/>
     <dataValidation type="list" allowBlank="1" showErrorMessage="1" sqref="A2:A13 A18:A52">

</xml_diff>